<commit_message>
Activa insumos sugeridos con horas estimadas en la matriz de PU
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UkotvK4ym43wx8Kw31Kuy
</commit_message>
<xml_diff>
--- a/Matriz_PU_Ingenieria_Estructural.xlsx
+++ b/Matriz_PU_Ingenieria_Estructural.xlsx
@@ -803,7 +803,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CÓMO USAR: en la columna A elige Sí/No para incluir o quitar cada insumo. Edita Cantidad y Costo Unitario (texto azul). Filas amarillas = insumos SUGERIDOS (valores estimados, ajustar). Los totales y gráficas se actualizan solos.</t>
+          <t>CÓMO USAR: en la columna A elige Sí/No para incluir o quitar cada insumo. Edita Cantidad y Costo Unitario (texto azul). Filas amarillas = insumos SUGERIDOS (horas y costos estimados por Claude, ya incluidos; quita con No los que no apliquen; el estudio de suelos queda en No por ser normalmente del cliente). Los totales y gráficas se actualizan solos.</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
@@ -1251,7 +1251,7 @@
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
@@ -1302,7 +1302,7 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
@@ -1353,7 +1353,7 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -1404,7 +1404,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
@@ -1455,7 +1455,7 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -1506,7 +1506,7 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
@@ -1557,7 +1557,7 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
@@ -1608,7 +1608,7 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
@@ -1800,7 +1800,7 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
@@ -1851,7 +1851,7 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
@@ -1902,7 +1902,7 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
@@ -2004,7 +2004,7 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B29" s="13" t="inlineStr">
@@ -2055,7 +2055,7 @@
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
@@ -2157,7 +2157,7 @@
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">

</xml_diff>